<commit_message>
Admin: edit data/shala-team.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/shala-team.xlsx
+++ b/data/shala-team.xlsx
@@ -459,7 +459,7 @@
         <v>Shala Vice Principal</v>
       </c>
       <c r="C3" t="str">
-        <v>Teachers</v>
+        <v>Shala Management</v>
       </c>
       <c r="D3" t="str">
         <v>assets/images/shala/team/manisha-rahatadkar.jpg</v>
@@ -511,7 +511,7 @@
         <v>Teacher</v>
       </c>
       <c r="C5" t="str">
-        <v>Shala Management</v>
+        <v>Teachers</v>
       </c>
       <c r="D5" t="str">
         <v>assets/images/shala/team/aaditi-dixit.jpg</v>

</xml_diff>